<commit_message>
Vimo: bo sung deposit_rate_tcbs_ipower_max bi thieu sau merge, chay lai pipeline
Doi chieu lai sau merge voi cron phat hien thieu 1 key schema
(deposit_rate_tcbs_ipower_max) chua duoc merge lai. Da bo sung va chay
lai fetch + report tren nen du lieu day du.

Luu y: sbv.gov.vn dang tam thoi chan IP (WAF rate-limit do test nhieu
lan trong phien lam viec nay) - cac chi so nguon SBV (credit_growth,
lai suat dieu hanh/lien ngan hang, OMO, tin phieu) chua co diem tuan
moi nhat, se tu cap nhat lai o lan chay theo lich tiep theo (khong lap
lai van de nay trong dieu kien binh thuong).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -675,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DY38"/>
+  <dimension ref="A1:DY42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1930,7 +1931,7 @@
         <v>26270</v>
       </c>
       <c r="P24" t="n">
-        <v>26250.54</v>
+        <v>26278.14</v>
       </c>
     </row>
     <row r="25">
@@ -3869,6 +3870,66 @@
       </c>
       <c r="DY38" t="n">
         <v>0.66</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>VN-Index P/E (ex-VIN)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>10.43598551518464</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>VN-Index P/B (ex-VIN)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>1.621001140786313</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>VN-Index P/E (headline, có VIN)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>12.38</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>VN-Index P/B (headline, có VIN)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>1.92</v>
       </c>
     </row>
   </sheetData>
@@ -4413,7 +4474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM5"/>
+  <dimension ref="A1:AN5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4455,6 +4516,7 @@
     <col width="12" customWidth="1" min="37" max="37"/>
     <col width="12" customWidth="1" min="38" max="38"/>
     <col width="12" customWidth="1" min="39" max="39"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4653,6 +4715,11 @@
           <t>2026-07-20</t>
         </is>
       </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4829,6 +4896,141 @@
       </c>
       <c r="AJ5" t="n">
         <v>-491.72</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>-1328.11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chỉ báo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Đơn vị</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2026-W30</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2026-W28</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lãi suất huy động 12T — Vietcombank (nhóm lớn)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lãi suất huy động 12T — VietinBank (nhóm lớn)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lãi suất huy động 12T — NamABank (nhóm nhỏ)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lãi suất huy động online 12 tháng — CAO NHẤT thị trường (đa ngân hàng)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lãi suất huy động online 12 tháng — TRUNG BÌNH thị trường (đa ngân hàng)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6.17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lãi suất iPower TCBS (cao nhất)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vimo: sua nhan quyet dinh qua manh, lam ro 2 khai niem ERP, lay lai du lieu SBV
- calc_decision_matrix: doi "Mua ty trong cao" -> "Nen mua vao" cho truong hop
  Re/Hap dan nhung vi mo chua tot (Scorecard am, nhieu nhom Xau) - "tang ty
  trong lon" chi danh rieng cho macro tot THAT SU (khong bi lai suat phu quyet)
- Them ghi chu phan biet 2 khai niem ERP (E/Y-Rf thuc te vs ERP Viet Nam ~7%
  gia dinh trong CAPM) o ca PDF va web, tranh nham lan khi hien thi cung trang
- sbv.gov.vn da het chan IP (WAF ret-limit truoc do) - da fetch lai thanh cong,
  bieu do lai suat lien ngan hang gio co du lieu thuc (khong con 1 diem)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -4912,7 +4912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5033,6 +5033,156 @@
         <v>9</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lãi suất tái cấp vốn (NHNN)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng 3 tháng</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>7.63</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng qua đêm (O/N)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2.97</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng 1 tuần</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng 2 tuần</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng 1 tháng</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6.65</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng 6 tháng</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lãi suất liên ngân hàng 9 tháng</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>9.26</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lãi suất OMO kỳ hạn 7 ngày (bơm thanh khoản)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Số ngày kể từ lần chào bán tín phiếu NHNN gần nhất (hút thanh khoản)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ngày</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>268</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Vimo: backfill co cau von dau tu Nha nuoc/Ngoai NN/FDI 10 quy (2024-Q1 den 2026-Q1), doc tu anh infographic NSO (OCR thu cong qua vision)
User tu tim va gui 9 link infographic NSO (nso.gov.vn/tin-tuc-thong-ke), phat hien du lieu that
nam trong ANH (khong phai text - trang HTML chi co menu/tin lien quan). Doc truc tiep panel anh
"DT-XNK-CPI"/"Thuong-mai" (panel dau tu/XNK/CPI) bang kha nang xem anh, lay dung so tuyet doi
Nha nuoc/Ngoai NN/FDI (nghin ty dong) cho tung ky, tinh % cho tung khu vuc - khop 100% voi
fdi_disbursed da co (doi chieu tung ky). investment_share_state/private/fdi: 1 diem -> 10 diem.
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -810,6 +810,69 @@
       </c>
       <c r="K14" t="n">
         <v>8.51</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cơ cấu vốn đầu tư — Khu vực Nhà nước</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>27.64</v>
+      </c>
+      <c r="K15" t="n">
+        <v>27.82</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cơ cấu vốn đầu tư — Khu vực ngoài Nhà nước (tư nhân)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>54.24</v>
+      </c>
+      <c r="K16" t="n">
+        <v>54.04</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cơ cấu vốn đầu tư — Khu vực FDI</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>18</v>
+      </c>
+      <c r="G17" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="K17" t="n">
+        <v>18.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vimo: chuyen omo_rate_7d tu SBV (tuan) sang VIRA (ngay that), backfill 11 diem tu ban tin da co
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -5257,7 +5257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR15"/>
+  <dimension ref="A1:AR16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -6194,6 +6194,51 @@
         <v>-1961.37</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lãi suất OMO kỳ hạn 7 ngày (bơm thanh khoản)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="AE16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Vimo: them so du OMO luu hanh (omo_outstanding_balance) tu ban tin VIRA, fix bug append VIRA lam sai thu tu period khi lap khoang trong
- omo_outstanding_balance moi: TON KHO thanh khoan NHNN dang luu hanh qua kenh cam co (khac
  omo_net_operation la DONG CHAY rong/ngay) - user 2026-07-30 chi ra ban tin VIRA co san so nay.
  Backfill 12 diem tu ban tin da co (08/07-29/07), giam dan 217,617 -> 144,342 ty dong, khop huong
  voi omo_net_operation da co (da so ngay hut rong)
- Fix bug goc: _append_point() chi noi vao CUOI series, nhung fetch_vira_bulletin() quet lui 10
  ngay MOI LAN chay co the lap duoc 1 ngay CU HON diem da luu (ban tin ra tre) - diem lap tre do
  bi noi SAI VI TRI (sau cac ngay moi hon) neu khong sort lai. Them buoc sort lai theo period cho
  moi key VIRA vua duoc ghi them trong lan chay do. Da fix luon thu tu sai san co cua
  omo_outstanding_balance (07-29 dung truoc 07-28 do loi nay khi lap khoang trong)
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -2141,7 +2141,7 @@
         <v>26270</v>
       </c>
       <c r="P24" t="n">
-        <v>26254</v>
+        <v>26183.58</v>
       </c>
     </row>
     <row r="25">
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>10.6592122785923</v>
+        <v>10.72887492722224</v>
       </c>
     </row>
     <row r="40">
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>1.655372223421629</v>
+        <v>1.666190810249435</v>
       </c>
     </row>
     <row r="41">
@@ -4124,7 +4124,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>12.43</v>
+        <v>12.38</v>
       </c>
     </row>
     <row r="42">
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>1.94</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="43">
@@ -5257,7 +5257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS16"/>
+  <dimension ref="A1:AT17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5305,6 +5305,7 @@
     <col width="12" customWidth="1" min="43" max="43"/>
     <col width="12" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5533,6 +5534,11 @@
           <t>2026-07-29</t>
         </is>
       </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5722,6 +5728,9 @@
       <c r="AS5" t="n">
         <v>-85.26000000000001</v>
       </c>
+      <c r="AT5" t="n">
+        <v>662.8200000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6279,6 +6288,57 @@
       </c>
       <c r="AS16" t="n">
         <v>4.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Số dư OMO đang lưu hành (kênh cầm cố)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tỷ đồng</t>
+        </is>
+      </c>
+      <c r="AE17" t="n">
+        <v>217617.1</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>211095.65</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>196090.35</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>187898.19</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>159415.82</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>192609.12</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>190047.26</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>181990.46</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>176178.38</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>163076.25</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>146020</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>144058.63</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>144342.34</v>
       </c>
     </row>
   </sheetData>
@@ -6467,7 +6527,7 @@
         <v>7.63</v>
       </c>
       <c r="E9" t="n">
-        <v>8.01</v>
+        <v>7.31</v>
       </c>
     </row>
     <row r="10">
@@ -6545,7 +6605,7 @@
         <v>7.8</v>
       </c>
       <c r="E14" t="n">
-        <v>8.48</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="15">
@@ -6599,7 +6659,7 @@
         <v>268</v>
       </c>
       <c r="E17" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vimo: backfill lich su VIRA ~120 ngay (OMO luu hanh len 4 thang, lai suat LNH + loi suat TPCP theo do), them bieu do rieng OMO luu hanh + bom/hut rong 2 truc Y; sua ID FRED sai cho EU CPI (con lai 4 chi bao EU/TQ chua tim duoc nguon thay the, note ro trong data)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5278,7 +5278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DR44"/>
+  <dimension ref="A1:FC44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5403,6 +5403,43 @@
     <col width="12" customWidth="1" min="120" max="120"/>
     <col width="12" customWidth="1" min="121" max="121"/>
     <col width="12" customWidth="1" min="122" max="122"/>
+    <col width="12" customWidth="1" min="123" max="123"/>
+    <col width="12" customWidth="1" min="124" max="124"/>
+    <col width="12" customWidth="1" min="125" max="125"/>
+    <col width="12" customWidth="1" min="126" max="126"/>
+    <col width="12" customWidth="1" min="127" max="127"/>
+    <col width="12" customWidth="1" min="128" max="128"/>
+    <col width="12" customWidth="1" min="129" max="129"/>
+    <col width="12" customWidth="1" min="130" max="130"/>
+    <col width="12" customWidth="1" min="131" max="131"/>
+    <col width="12" customWidth="1" min="132" max="132"/>
+    <col width="12" customWidth="1" min="133" max="133"/>
+    <col width="12" customWidth="1" min="134" max="134"/>
+    <col width="12" customWidth="1" min="135" max="135"/>
+    <col width="12" customWidth="1" min="136" max="136"/>
+    <col width="12" customWidth="1" min="137" max="137"/>
+    <col width="12" customWidth="1" min="138" max="138"/>
+    <col width="12" customWidth="1" min="139" max="139"/>
+    <col width="12" customWidth="1" min="140" max="140"/>
+    <col width="12" customWidth="1" min="141" max="141"/>
+    <col width="12" customWidth="1" min="142" max="142"/>
+    <col width="12" customWidth="1" min="143" max="143"/>
+    <col width="12" customWidth="1" min="144" max="144"/>
+    <col width="12" customWidth="1" min="145" max="145"/>
+    <col width="12" customWidth="1" min="146" max="146"/>
+    <col width="12" customWidth="1" min="147" max="147"/>
+    <col width="12" customWidth="1" min="148" max="148"/>
+    <col width="12" customWidth="1" min="149" max="149"/>
+    <col width="12" customWidth="1" min="150" max="150"/>
+    <col width="12" customWidth="1" min="151" max="151"/>
+    <col width="12" customWidth="1" min="152" max="152"/>
+    <col width="12" customWidth="1" min="153" max="153"/>
+    <col width="12" customWidth="1" min="154" max="154"/>
+    <col width="12" customWidth="1" min="155" max="155"/>
+    <col width="12" customWidth="1" min="156" max="156"/>
+    <col width="12" customWidth="1" min="157" max="157"/>
+    <col width="12" customWidth="1" min="158" max="158"/>
+    <col width="12" customWidth="1" min="159" max="159"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6014,6 +6051,191 @@
       <c r="DR1" t="inlineStr">
         <is>
           <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="DS1" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="DT1" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="DU1" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="DV1" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="DW1" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="DX1" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="DY1" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="DZ1" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="EA1" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="EB1" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="EC1" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="ED1" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="EE1" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="EF1" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="EG1" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="EI1" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="EJ1" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="EK1" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="EM1" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="EN1" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="EO1" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="EP1" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="EQ1" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="ER1" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="ES1" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="ET1" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="EU1" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="EV1" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="EW1" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="EX1" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="EY1" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="EZ1" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="FA1" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="FB1" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="FC1" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vimo: them 2 bieu do phai sinh tu credit_balance_total - tang truong du no tin dung YoY THAT theo thang (khac credit_growth SBV von la so voi dau nam), va ty le Tin dung/GDP danh nghia (World Bank, chi bao don bay tin dung kinh dien BIS/IMF)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DZ52"/>
+  <dimension ref="A1:DZ54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4706,6 +4706,582 @@
         <v>45.82</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Tăng trưởng dư nợ tín dụng toàn nền kinh tế YoY (theo tháng)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>19.22</v>
+      </c>
+      <c r="G53" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="H53" t="n">
+        <v>20.24</v>
+      </c>
+      <c r="I53" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="J53" t="n">
+        <v>19.83</v>
+      </c>
+      <c r="K53" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="L53" t="n">
+        <v>18.24</v>
+      </c>
+      <c r="M53" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="N53" t="n">
+        <v>18.23</v>
+      </c>
+      <c r="BA53" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="BB53" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="BC53" t="n">
+        <v>13.45</v>
+      </c>
+      <c r="BD53" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="BE53" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="BF53" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="BG53" t="n">
+        <v>13.28</v>
+      </c>
+      <c r="BH53" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="BI53" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="BJ53" t="n">
+        <v>12.73</v>
+      </c>
+      <c r="BK53" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="BL53" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="BM53" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="BN53" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="BO53" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="BP53" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="BQ53" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="BR53" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="BS53" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="BT53" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="BU53" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="BV53" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="BW53" t="n">
+        <v>11</v>
+      </c>
+      <c r="BX53" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="BY53" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="BZ53" t="n">
+        <v>12.71</v>
+      </c>
+      <c r="CA53" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="CB53" t="n">
+        <v>15.21</v>
+      </c>
+      <c r="CC53" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="CD53" t="n">
+        <v>15.19</v>
+      </c>
+      <c r="CE53" t="n">
+        <v>15.26</v>
+      </c>
+      <c r="CF53" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="CG53" t="n">
+        <v>14.07</v>
+      </c>
+      <c r="CH53" t="n">
+        <v>14.24</v>
+      </c>
+      <c r="CI53" t="n">
+        <v>14.64</v>
+      </c>
+      <c r="CJ53" t="n">
+        <v>13.61</v>
+      </c>
+      <c r="CK53" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="CL53" t="n">
+        <v>15.86</v>
+      </c>
+      <c r="CM53" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="CN53" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="CO53" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="CP53" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="CQ53" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="CR53" t="n">
+        <v>16.28</v>
+      </c>
+      <c r="CS53" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="CT53" t="n">
+        <v>16.59</v>
+      </c>
+      <c r="CU53" t="n">
+        <v>14.84</v>
+      </c>
+      <c r="CV53" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="CW53" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="CX53" t="n">
+        <v>12.17</v>
+      </c>
+      <c r="CY53" t="n">
+        <v>10.52</v>
+      </c>
+      <c r="CZ53" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="DA53" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="DB53" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="DC53" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="DD53" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="DE53" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="DF53" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="DG53" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="DH53" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="DI53" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="DJ53" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="DK53" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="DL53" t="n">
+        <v>12.67</v>
+      </c>
+      <c r="DM53" t="n">
+        <v>13.97</v>
+      </c>
+      <c r="DN53" t="n">
+        <v>15.28</v>
+      </c>
+      <c r="DO53" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="DP53" t="n">
+        <v>15.67</v>
+      </c>
+      <c r="DQ53" t="n">
+        <v>16.08</v>
+      </c>
+      <c r="DR53" t="n">
+        <v>16.69</v>
+      </c>
+      <c r="DS53" t="n">
+        <v>16.56</v>
+      </c>
+      <c r="DT53" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="DU53" t="n">
+        <v>16.52</v>
+      </c>
+      <c r="DV53" t="n">
+        <v>16.84</v>
+      </c>
+      <c r="DW53" t="n">
+        <v>17.91</v>
+      </c>
+      <c r="DX53" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="DY53" t="n">
+        <v>18.75</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Tỷ lệ Tín dụng / GDP danh nghĩa</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>133.59</v>
+      </c>
+      <c r="G54" t="n">
+        <v>140.16</v>
+      </c>
+      <c r="H54" t="n">
+        <v>142.03</v>
+      </c>
+      <c r="I54" t="n">
+        <v>146.45</v>
+      </c>
+      <c r="J54" t="n">
+        <v>146.45</v>
+      </c>
+      <c r="K54" t="n">
+        <v>149.34</v>
+      </c>
+      <c r="L54" t="n">
+        <v>149.34</v>
+      </c>
+      <c r="M54" t="n">
+        <v>151.37</v>
+      </c>
+      <c r="N54" t="n">
+        <v>153.37</v>
+      </c>
+      <c r="AO54" t="n">
+        <v>91.18000000000001</v>
+      </c>
+      <c r="AP54" t="n">
+        <v>91.54000000000001</v>
+      </c>
+      <c r="AQ54" t="n">
+        <v>93.53</v>
+      </c>
+      <c r="AR54" t="n">
+        <v>94.94</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>95.92</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="AU54" t="n">
+        <v>97.62</v>
+      </c>
+      <c r="AV54" t="n">
+        <v>98.45</v>
+      </c>
+      <c r="AW54" t="n">
+        <v>99.67</v>
+      </c>
+      <c r="AX54" t="n">
+        <v>100.42</v>
+      </c>
+      <c r="AY54" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="AZ54" t="n">
+        <v>102.88</v>
+      </c>
+      <c r="BA54" t="n">
+        <v>95.34999999999999</v>
+      </c>
+      <c r="BB54" t="n">
+        <v>94.56</v>
+      </c>
+      <c r="BC54" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="BD54" t="n">
+        <v>97.73999999999999</v>
+      </c>
+      <c r="BE54" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="BF54" t="n">
+        <v>100.45</v>
+      </c>
+      <c r="BG54" t="n">
+        <v>100.57</v>
+      </c>
+      <c r="BH54" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="BI54" t="n">
+        <v>102.36</v>
+      </c>
+      <c r="BJ54" t="n">
+        <v>102.95</v>
+      </c>
+      <c r="BK54" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="BL54" t="n">
+        <v>106.33</v>
+      </c>
+      <c r="BM54" t="n">
+        <v>101.98</v>
+      </c>
+      <c r="BN54" t="n">
+        <v>102.05</v>
+      </c>
+      <c r="BO54" t="n">
+        <v>103.21</v>
+      </c>
+      <c r="BP54" t="n">
+        <v>103.32</v>
+      </c>
+      <c r="BQ54" t="n">
+        <v>103.91</v>
+      </c>
+      <c r="BR54" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="BS54" t="n">
+        <v>106</v>
+      </c>
+      <c r="BT54" t="n">
+        <v>106.79</v>
+      </c>
+      <c r="BU54" t="n">
+        <v>108.08</v>
+      </c>
+      <c r="BV54" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="BW54" t="n">
+        <v>110.45</v>
+      </c>
+      <c r="BX54" t="n">
+        <v>114.27</v>
+      </c>
+      <c r="BY54" t="n">
+        <v>109.13</v>
+      </c>
+      <c r="BZ54" t="n">
+        <v>109.02</v>
+      </c>
+      <c r="CA54" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="CB54" t="n">
+        <v>112.82</v>
+      </c>
+      <c r="CC54" t="n">
+        <v>113.67</v>
+      </c>
+      <c r="CD54" t="n">
+        <v>115.29</v>
+      </c>
+      <c r="CE54" t="n">
+        <v>115.8</v>
+      </c>
+      <c r="CF54" t="n">
+        <v>116.38</v>
+      </c>
+      <c r="CG54" t="n">
+        <v>116.84</v>
+      </c>
+      <c r="CH54" t="n">
+        <v>117.8</v>
+      </c>
+      <c r="CI54" t="n">
+        <v>120.01</v>
+      </c>
+      <c r="CJ54" t="n">
+        <v>123.05</v>
+      </c>
+      <c r="CK54" t="n">
+        <v>111.43</v>
+      </c>
+      <c r="CL54" t="n">
+        <v>111.43</v>
+      </c>
+      <c r="CM54" t="n">
+        <v>115.03</v>
+      </c>
+      <c r="CN54" t="n">
+        <v>116.4</v>
+      </c>
+      <c r="CO54" t="n">
+        <v>117.33</v>
+      </c>
+      <c r="CP54" t="n">
+        <v>118.78</v>
+      </c>
+      <c r="CQ54" t="n">
+        <v>118.91</v>
+      </c>
+      <c r="CR54" t="n">
+        <v>119.37</v>
+      </c>
+      <c r="CS54" t="n">
+        <v>120.54</v>
+      </c>
+      <c r="CT54" t="n">
+        <v>121.16</v>
+      </c>
+      <c r="CU54" t="n">
+        <v>121.58</v>
+      </c>
+      <c r="CV54" t="n">
+        <v>123.94</v>
+      </c>
+      <c r="CW54" t="n">
+        <v>115.68</v>
+      </c>
+      <c r="CX54" t="n">
+        <v>116.54</v>
+      </c>
+      <c r="CY54" t="n">
+        <v>118.54</v>
+      </c>
+      <c r="CZ54" t="n">
+        <v>119.05</v>
+      </c>
+      <c r="DA54" t="n">
+        <v>119.33</v>
+      </c>
+      <c r="DB54" t="n">
+        <v>121.02</v>
+      </c>
+      <c r="DC54" t="n">
+        <v>120.81</v>
+      </c>
+      <c r="DD54" t="n">
+        <v>121.99</v>
+      </c>
+      <c r="DE54" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="DF54" t="n">
+        <v>124.12</v>
+      </c>
+      <c r="DG54" t="n">
+        <v>126.17</v>
+      </c>
+      <c r="DH54" t="n">
+        <v>131.49</v>
+      </c>
+      <c r="DI54" t="n">
+        <v>117.08</v>
+      </c>
+      <c r="DJ54" t="n">
+        <v>117</v>
+      </c>
+      <c r="DK54" t="n">
+        <v>119.56</v>
+      </c>
+      <c r="DL54" t="n">
+        <v>120.26</v>
+      </c>
+      <c r="DM54" t="n">
+        <v>121.93</v>
+      </c>
+      <c r="DN54" t="n">
+        <v>125.07</v>
+      </c>
+      <c r="DO54" t="n">
+        <v>124.87</v>
+      </c>
+      <c r="DP54" t="n">
+        <v>126.51</v>
+      </c>
+      <c r="DQ54" t="n">
+        <v>128.63</v>
+      </c>
+      <c r="DR54" t="n">
+        <v>129.84</v>
+      </c>
+      <c r="DS54" t="n">
+        <v>131.85</v>
+      </c>
+      <c r="DT54" t="n">
+        <v>135.67</v>
+      </c>
+      <c r="DU54" t="n">
+        <v>122.22</v>
+      </c>
+      <c r="DV54" t="n">
+        <v>122.48</v>
+      </c>
+      <c r="DW54" t="n">
+        <v>126.3</v>
+      </c>
+      <c r="DX54" t="n">
+        <v>128.01</v>
+      </c>
+      <c r="DY54" t="n">
+        <v>129.72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4717,7 +5293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4968,6 +5544,48 @@
       </c>
       <c r="M6" t="n">
         <v>-3.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GDP danh nghĩa Việt Nam (theo năm)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tỷ VND</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6293904.55</v>
+      </c>
+      <c r="D7" t="n">
+        <v>7009042.13</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7707200.29</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8044385.73</v>
+      </c>
+      <c r="G7" t="n">
+        <v>8487475.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>9621371.82</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10319058.87</v>
+      </c>
+      <c r="J7" t="n">
+        <v>11510328.92</v>
+      </c>
+      <c r="K7" t="n">
+        <v>12847571.22</v>
+      </c>
+      <c r="M7" t="n">
+        <v>5639401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vimo: them deposit_balance_total (VBMA, Tien gui TCKT + dan cu, cung file CSV voi M2) va deposit_growth_yoy_monthly phai sinh - dap ung yeu cau doi chieu tang truong huy dong tu data.vietnambiz.vn; ghep 3 duong tin dung/M2/huy dong YoY vao 1 chart; bump cache-bust v5->v6
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo quý" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tháng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo năm" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DZ54"/>
+  <dimension ref="A1:DZ56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5280,6 +5280,528 @@
       </c>
       <c r="DY54" t="n">
         <v>129.72</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tổng huy động vốn toàn nền kinh tế</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>tỷ VND</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>15798887</v>
+      </c>
+      <c r="D55" t="n">
+        <v>15725450</v>
+      </c>
+      <c r="E55" t="n">
+        <v>15959293</v>
+      </c>
+      <c r="F55" t="n">
+        <v>16182630</v>
+      </c>
+      <c r="G55" t="n">
+        <v>15909571</v>
+      </c>
+      <c r="H55" t="n">
+        <v>16064674</v>
+      </c>
+      <c r="I55" t="n">
+        <v>16515887</v>
+      </c>
+      <c r="J55" t="n">
+        <v>16461627</v>
+      </c>
+      <c r="K55" t="n">
+        <v>16415112</v>
+      </c>
+      <c r="L55" t="n">
+        <v>16575580</v>
+      </c>
+      <c r="M55" t="n">
+        <v>16793661</v>
+      </c>
+      <c r="AZ55" t="n">
+        <v>7717980</v>
+      </c>
+      <c r="BA55" t="n">
+        <v>7729722</v>
+      </c>
+      <c r="BB55" t="n">
+        <v>7784927</v>
+      </c>
+      <c r="BC55" t="n">
+        <v>7886700</v>
+      </c>
+      <c r="BD55" t="n">
+        <v>7925247</v>
+      </c>
+      <c r="BE55" t="n">
+        <v>8102385</v>
+      </c>
+      <c r="BF55" t="n">
+        <v>8233716</v>
+      </c>
+      <c r="BG55" t="n">
+        <v>8249223</v>
+      </c>
+      <c r="BH55" t="n">
+        <v>8283755</v>
+      </c>
+      <c r="BI55" t="n">
+        <v>8421336</v>
+      </c>
+      <c r="BJ55" t="n">
+        <v>8471733</v>
+      </c>
+      <c r="BK55" t="n">
+        <v>8567206</v>
+      </c>
+      <c r="BL55" t="n">
+        <v>8792649</v>
+      </c>
+      <c r="BM55" t="n">
+        <v>8739395</v>
+      </c>
+      <c r="BN55" t="n">
+        <v>8789582</v>
+      </c>
+      <c r="BO55" t="n">
+        <v>8820899</v>
+      </c>
+      <c r="BP55" t="n">
+        <v>8798935</v>
+      </c>
+      <c r="BQ55" t="n">
+        <v>8996217</v>
+      </c>
+      <c r="BR55" t="n">
+        <v>9209997</v>
+      </c>
+      <c r="BS55" t="n">
+        <v>9219381</v>
+      </c>
+      <c r="BT55" t="n">
+        <v>9327466</v>
+      </c>
+      <c r="BU55" t="n">
+        <v>9483045</v>
+      </c>
+      <c r="BV55" t="n">
+        <v>9541346</v>
+      </c>
+      <c r="BW55" t="n">
+        <v>9697185</v>
+      </c>
+      <c r="BX55" t="n">
+        <v>10019859</v>
+      </c>
+      <c r="BY55" t="n">
+        <v>9983024</v>
+      </c>
+      <c r="BZ55" t="n">
+        <v>9979753</v>
+      </c>
+      <c r="CA55" t="n">
+        <v>10169387</v>
+      </c>
+      <c r="CB55" t="n">
+        <v>10240129</v>
+      </c>
+      <c r="CC55" t="n">
+        <v>10312681</v>
+      </c>
+      <c r="CD55" t="n">
+        <v>10404260</v>
+      </c>
+      <c r="CE55" t="n">
+        <v>10379604</v>
+      </c>
+      <c r="CF55" t="n">
+        <v>10437766</v>
+      </c>
+      <c r="CG55" t="n">
+        <v>10549000</v>
+      </c>
+      <c r="CH55" t="n">
+        <v>10550758</v>
+      </c>
+      <c r="CI55" t="n">
+        <v>10680562</v>
+      </c>
+      <c r="CJ55" t="n">
+        <v>10945849</v>
+      </c>
+      <c r="CK55" t="n">
+        <v>10980777</v>
+      </c>
+      <c r="CL55" t="n">
+        <v>11096605</v>
+      </c>
+      <c r="CM55" t="n">
+        <v>11339315</v>
+      </c>
+      <c r="CN55" t="n">
+        <v>11327466</v>
+      </c>
+      <c r="CO55" t="n">
+        <v>11375944</v>
+      </c>
+      <c r="CP55" t="n">
+        <v>11468408</v>
+      </c>
+      <c r="CQ55" t="n">
+        <v>11394485</v>
+      </c>
+      <c r="CR55" t="n">
+        <v>11314657</v>
+      </c>
+      <c r="CS55" t="n">
+        <v>11420867</v>
+      </c>
+      <c r="CT55" t="n">
+        <v>11426633</v>
+      </c>
+      <c r="CU55" t="n">
+        <v>11553571</v>
+      </c>
+      <c r="CV55" t="n">
+        <v>11819462</v>
+      </c>
+      <c r="CW55" t="n">
+        <v>11748113</v>
+      </c>
+      <c r="CX55" t="n">
+        <v>11795598</v>
+      </c>
+      <c r="CY55" t="n">
+        <v>11944562</v>
+      </c>
+      <c r="CZ55" t="n">
+        <v>11987757</v>
+      </c>
+      <c r="DA55" t="n">
+        <v>12096031</v>
+      </c>
+      <c r="DB55" t="n">
+        <v>12366810</v>
+      </c>
+      <c r="DC55" t="n">
+        <v>12299300</v>
+      </c>
+      <c r="DD55" t="n">
+        <v>12446524</v>
+      </c>
+      <c r="DE55" t="n">
+        <v>12679812</v>
+      </c>
+      <c r="DF55" t="n">
+        <v>12703788</v>
+      </c>
+      <c r="DG55" t="n">
+        <v>12855295</v>
+      </c>
+      <c r="DH55" t="n">
+        <v>13374474</v>
+      </c>
+      <c r="DI55" t="n">
+        <v>13174612</v>
+      </c>
+      <c r="DJ55" t="n">
+        <v>13160231</v>
+      </c>
+      <c r="DK55" t="n">
+        <v>13303208</v>
+      </c>
+      <c r="DL55" t="n">
+        <v>13292066</v>
+      </c>
+      <c r="DM55" t="n">
+        <v>13424014</v>
+      </c>
+      <c r="DN55" t="n">
+        <v>13724841</v>
+      </c>
+      <c r="DO55" t="n">
+        <v>13607169</v>
+      </c>
+      <c r="DP55" t="n">
+        <v>13763231</v>
+      </c>
+      <c r="DQ55" t="n">
+        <v>14034142</v>
+      </c>
+      <c r="DR55" t="n">
+        <v>14136939</v>
+      </c>
+      <c r="DS55" t="n">
+        <v>14270065</v>
+      </c>
+      <c r="DT55" t="n">
+        <v>14732270</v>
+      </c>
+      <c r="DU55" t="n">
+        <v>14621852</v>
+      </c>
+      <c r="DV55" t="n">
+        <v>14728372</v>
+      </c>
+      <c r="DW55" t="n">
+        <v>14990204</v>
+      </c>
+      <c r="DX55" t="n">
+        <v>15162767</v>
+      </c>
+      <c r="DY55" t="n">
+        <v>15344564</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tăng trưởng huy động vốn toàn nền kinh tế YoY (theo tháng)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="D56" t="n">
+        <v>15.57</v>
+      </c>
+      <c r="E56" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="F56" t="n">
+        <v>15.31</v>
+      </c>
+      <c r="G56" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="H56" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="I56" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="J56" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="K56" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="L56" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="M56" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="BL56" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="BM56" t="n">
+        <v>13.06</v>
+      </c>
+      <c r="BN56" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="BO56" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="BP56" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="BQ56" t="n">
+        <v>11.03</v>
+      </c>
+      <c r="BR56" t="n">
+        <v>11.86</v>
+      </c>
+      <c r="BS56" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="BT56" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="BU56" t="n">
+        <v>12.61</v>
+      </c>
+      <c r="BV56" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="BW56" t="n">
+        <v>13.19</v>
+      </c>
+      <c r="BX56" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="BY56" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="BZ56" t="n">
+        <v>13.54</v>
+      </c>
+      <c r="CA56" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="CB56" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="CC56" t="n">
+        <v>14.63</v>
+      </c>
+      <c r="CD56" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="CE56" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="CF56" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="CG56" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="CH56" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="CI56" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="CJ56" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="CK56" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="CL56" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="CM56" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="CN56" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="CO56" t="n">
+        <v>10.31</v>
+      </c>
+      <c r="CP56" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="CQ56" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="CR56" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="CS56" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="CT56" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="CU56" t="n">
+        <v>8.17</v>
+      </c>
+      <c r="CV56" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="CW56" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="CX56" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="CY56" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="CZ56" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="DA56" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="DB56" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="DC56" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="DD56" t="n">
+        <v>10</v>
+      </c>
+      <c r="DE56" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="DF56" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="DG56" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="DH56" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="DI56" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="DJ56" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="DK56" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="DL56" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="DM56" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="DN56" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="DO56" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="DP56" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="DQ56" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="DR56" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="DS56" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="DT56" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="DU56" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="DV56" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="DW56" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="DX56" t="n">
+        <v>14.07</v>
+      </c>
+      <c r="DY56" t="n">
+        <v>14.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vimo: fix bug tiem an - fetch_vbma_cpi_contribution() da duoc goi san trong pipeline nhung 5 key cpi_contrib_* chua co trong schema, se KeyError ngay khi VBMA tra du lieu that; them schema + du lieu that (78 diem/nhom tu T1/2020), dua vao Bang giam sat theo yeu cau user (doi chieu anh CPI theo nhom hang)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DZ56"/>
+  <dimension ref="A1:DZ61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5802,6 +5802,1236 @@
       </c>
       <c r="DY56" t="n">
         <v>14.31</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Đóng góp vào lạm phát — nhóm Thực phẩm</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>điểm %</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I57" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J57" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="N57" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="O57" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="BM57" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="BN57" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="BO57" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="BP57" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="BQ57" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="BR57" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="BS57" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="BT57" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="BU57" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="BV57" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="BW57" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="BX57" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BY57" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="BZ57" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CA57" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="CB57" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="CC57" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="CD57" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="CE57" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="CF57" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="CG57" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="CH57" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="CI57" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="CJ57" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="CK57" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="CL57" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="CM57" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="CN57" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="CO57" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="CP57" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="CQ57" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR57" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="CS57" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="CT57" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="CU57" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="CV57" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="CW57" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="CX57" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="CY57" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="CZ57" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="DA57" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="DB57" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="DC57" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="DD57" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="DE57" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="DF57" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="DG57" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH57" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="DI57" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="DJ57" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="DK57" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="DL57" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="DM57" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="DN57" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="DO57" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="DP57" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="DQ57" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="DR57" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="DS57" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="DT57" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="DU57" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="DV57" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="DW57" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="DX57" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="DY57" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Đóng góp vào lạm phát — nhóm Nhà, điện, nước</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>điểm %</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G58" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K58" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="M58" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N58" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="O58" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="BM58" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="BN58" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="BO58" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="BP58" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="BQ58" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="BR58" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BS58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="BT58" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="BU58" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BV58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="BW58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="BX58" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="BY58" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="BZ58" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="CA58" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="CB58" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="CC58" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="CD58" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="CE58" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="CF58" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="CG58" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="CH58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="CI58" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="CJ58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="CK58" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="CL58" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="CM58" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="CN58" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="CO58" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="CP58" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="CQ58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="CR58" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="CS58" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="CT58" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="CU58" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="CV58" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="CW58" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="CX58" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="CY58" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="CZ58" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="DA58" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="DB58" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="DC58" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="DD58" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="DE58" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="DF58" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="DG58" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="DH58" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="DI58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="DJ58" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="DK58" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="DL58" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="DM58" t="n">
+        <v>1</v>
+      </c>
+      <c r="DN58" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="DO58" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="DP58" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="DQ58" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="DR58" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="DS58" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="DT58" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="DU58" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="DV58" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="DW58" t="n">
+        <v>1</v>
+      </c>
+      <c r="DX58" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="DY58" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Đóng góp vào lạm phát — nhóm Y tế</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>điểm %</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="BM59" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="BN59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BO59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BP59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BQ59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BR59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BS59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BT59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BU59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BV59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BW59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BX59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="BY59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BZ59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CA59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CB59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CC59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CD59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CE59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CF59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CG59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CH59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CI59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CJ59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CK59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CL59" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="CM59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="CN59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="CO59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="CP59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="CQ59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="CR59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CS59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CT59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CU59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CV59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CW59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CX59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CY59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="CZ59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DA59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DB59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DC59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DD59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DE59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DF59" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="DG59" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="DH59" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="DI59" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="DJ59" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="DK59" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="DL59" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DM59" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DN59" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="DO59" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="DP59" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="DQ59" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="DR59" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="DS59" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="DT59" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="DU59" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="DV59" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="DW59" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="DX59" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="DY59" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Đóng góp vào lạm phát — nhóm Vận tải</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>điểm %</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="D60" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="J60" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="K60" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="L60" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="M60" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="N60" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="BM60" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="BN60" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BO60" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="BP60" t="n">
+        <v>-1.89</v>
+      </c>
+      <c r="BQ60" t="n">
+        <v>-2.26</v>
+      </c>
+      <c r="BR60" t="n">
+        <v>-1.67</v>
+      </c>
+      <c r="BS60" t="n">
+        <v>-1.36</v>
+      </c>
+      <c r="BT60" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="BU60" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="BV60" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="BW60" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="BX60" t="n">
+        <v>-1.13</v>
+      </c>
+      <c r="BY60" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="BZ60" t="n">
+        <v>-0.63</v>
+      </c>
+      <c r="CA60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="CB60" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="CC60" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="CD60" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="CE60" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="CF60" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="CG60" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="CH60" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="CI60" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ60" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="CK60" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="CL60" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="CM60" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="CN60" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="CO60" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="CP60" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="CQ60" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="CR60" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="CS60" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="CT60" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="CU60" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="CV60" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="CW60" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX60" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="CY60" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="CZ60" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="DA60" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="DB60" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="DC60" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="DD60" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="DE60" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="DF60" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="DG60" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="DH60" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="DI60" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="DJ60" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="DK60" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="DL60" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="DM60" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="DN60" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="DO60" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="DP60" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="DQ60" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="DR60" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="DS60" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="DT60" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="DU60" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="DV60" t="n">
+        <v>-0.27</v>
+      </c>
+      <c r="DW60" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="DX60" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="DY60" t="n">
+        <v>-0.55</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Đóng góp vào lạm phát — nhóm Khác</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>điểm %</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="M61" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="N61" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="O61" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="BM61" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="BN61" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="BO61" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="BP61" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="BQ61" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="BR61" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BS61" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="BT61" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="BU61" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="BV61" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="BW61" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="BX61" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="BY61" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="BZ61" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="CA61" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CB61" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="CC61" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="CD61" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="CE61" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="CF61" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="CG61" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="CH61" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="CI61" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="CJ61" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="CK61" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="CL61" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="CM61" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="CN61" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="CO61" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="CP61" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="CQ61" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="CR61" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="CS61" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="CT61" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="CU61" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="CV61" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="CW61" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="CX61" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="CY61" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="CZ61" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="DA61" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="DB61" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="DC61" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="DD61" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="DE61" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="DF61" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="DG61" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH61" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="DI61" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="DJ61" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="DK61" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="DL61" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="DM61" t="n">
+        <v>1</v>
+      </c>
+      <c r="DN61" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="DO61" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="DP61" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="DQ61" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="DR61" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="DS61" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="DT61" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="DU61" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="DV61" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="DW61" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="DX61" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="DY61" t="n">
+        <v>0.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backfill ALM ngan hang — 2025-Q2 — 2026-08-31
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Lũy kế (H1-9M-FY)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Theo ngày" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Theo tuần" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ALM_NganHang_Raw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29894,4 +29895,4566 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S79"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Ma</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Ky</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Trang thai</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Va tu ky</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Tong tai san (ty)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>VCSH (ty)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NII (ty)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Tien gui KH (ty)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Liquid Assets (ty)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Gap lai suat rong &lt;=1nam (ty)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Gap lai suat/TTS (%)</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Gap thanh khoan rong &lt;=1thang (ty)</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Gap thanh khoan/TTS (%)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Stress NII +100bp (ty)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Stress NII +100bp/NII (%)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Che phu rut -10% tien gui (lan)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Nguon (tieu de)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Nguon (url)</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Cap nhat luc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>183753.294</v>
+      </c>
+      <c r="F2" t="n">
+        <v>14356.754</v>
+      </c>
+      <c r="G2" t="n">
+        <v>832.067</v>
+      </c>
+      <c r="H2" t="n">
+        <v>89748.55100000001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>52951.186</v>
+      </c>
+      <c r="J2" t="n">
+        <v>58964.887</v>
+      </c>
+      <c r="K2" t="n">
+        <v>32.089</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-6979.3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-3.798</v>
+      </c>
+      <c r="N2" t="n">
+        <v>196</v>
+      </c>
+      <c r="O2" t="n">
+        <v>23.556</v>
+      </c>
+      <c r="P2" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00032098765432098763ngn-hng-tmcp-an-bnh29042025-000000bo-co-ti-chnh-qu-1-2025.pdf</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:54:52+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>204916.735</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15373.082</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1504.021</v>
+      </c>
+      <c r="H3" t="n">
+        <v>123056.541</v>
+      </c>
+      <c r="I3" t="n">
+        <v>52527.126</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>4.269</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00012345679012345679ngn-hng-tmcp-an-bnh04092025-000000bo-co-ti-chnh-bn-nin-2025_1_0945.pdf</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:41:33+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>220494.731</v>
+      </c>
+      <c r="F4" t="n">
+        <v>16800.695</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1708.898</v>
+      </c>
+      <c r="H4" t="n">
+        <v>133411.372</v>
+      </c>
+      <c r="I4" t="n">
+        <v>47661.015</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-2072.081999999995</v>
+      </c>
+      <c r="K4" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>124</v>
+      </c>
+      <c r="O4" t="n">
+        <v>7.256</v>
+      </c>
+      <c r="P4" t="n">
+        <v>3.572</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/_604250_Bao_cao_tai_chinh_nam_2025_1775705238.pdf</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:05:32+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ACB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>891674.563</v>
+      </c>
+      <c r="F5" t="n">
+        <v>87074.577</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6358.865</v>
+      </c>
+      <c r="H5" t="n">
+        <v>550375.02</v>
+      </c>
+      <c r="I5" t="n">
+        <v>148662.648</v>
+      </c>
+      <c r="J5" t="n">
+        <v>252303.897</v>
+      </c>
+      <c r="K5" t="n">
+        <v>28.296</v>
+      </c>
+      <c r="L5" t="n">
+        <v>13417.335</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1419</v>
+      </c>
+      <c r="O5" t="n">
+        <v>22.315</v>
+      </c>
+      <c r="P5" t="n">
+        <v>2.701</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/ACB_Baocaotaichinh_Q1_2025_Hopnhat_13052025091456.pdf</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:55:57+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ACB</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>933541.42</v>
+      </c>
+      <c r="F6" t="n">
+        <v>87210.629</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6683.848</v>
+      </c>
+      <c r="H6" t="n">
+        <v>567406.86</v>
+      </c>
+      <c r="I6" t="n">
+        <v>137553.297</v>
+      </c>
+      <c r="J6" t="n">
+        <v>85041.65799999997</v>
+      </c>
+      <c r="K6" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-198166.713</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-21.227</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1288</v>
+      </c>
+      <c r="O6" t="n">
+        <v>19.27</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2.424</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/ACB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_19092025164217.pdf</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:43:25+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ACB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:05:37+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BAB</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>175365.541</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12075.66</v>
+      </c>
+      <c r="G8" t="n">
+        <v>873.981</v>
+      </c>
+      <c r="H8" t="n">
+        <v>124794.49</v>
+      </c>
+      <c r="I8" t="n">
+        <v>20918.596</v>
+      </c>
+      <c r="J8" t="n">
+        <v>19828.909</v>
+      </c>
+      <c r="K8" t="n">
+        <v>11.307</v>
+      </c>
+      <c r="L8" t="n">
+        <v>12897.777</v>
+      </c>
+      <c r="M8" t="n">
+        <v>7.355</v>
+      </c>
+      <c r="N8" t="n">
+        <v>274</v>
+      </c>
+      <c r="O8" t="n">
+        <v>31.351</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1.676</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/BAB_25Q1_BCTC_HN_07052025141647.pdf</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2026-08-31T09:57:27+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BAB</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>184957.884</v>
+      </c>
+      <c r="F9" t="n">
+        <v>12204.005</v>
+      </c>
+      <c r="G9" t="n">
+        <v>892.223</v>
+      </c>
+      <c r="H9" t="n">
+        <v>131084.67</v>
+      </c>
+      <c r="I9" t="n">
+        <v>27025.886</v>
+      </c>
+      <c r="J9" t="n">
+        <v>18047.83</v>
+      </c>
+      <c r="K9" t="n">
+        <v>9.757999999999999</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10385.428</v>
+      </c>
+      <c r="M9" t="n">
+        <v>5.615</v>
+      </c>
+      <c r="N9" t="n">
+        <v>303</v>
+      </c>
+      <c r="O9" t="n">
+        <v>33.96</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2.062</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00015520282186948853ngn-hng-tmcp-bc-30072025-000000bo-co-ti-chnh-qu-2-2025_3_0910.pdf</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:44:48+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BAB</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>195820.302</v>
+      </c>
+      <c r="F10" t="n">
+        <v>13308.904</v>
+      </c>
+      <c r="G10" t="n">
+        <v>979.295</v>
+      </c>
+      <c r="H10" t="n">
+        <v>127023.635</v>
+      </c>
+      <c r="I10" t="n">
+        <v>28133.503</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1734.546</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2.215</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/_604687_Bao_cao_tai_chinh_nam_2025_1774883201.pdf</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:08:17+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BID</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:01:27+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BID</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:50:13+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BID</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:08:21+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BVB</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>110118.131</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6219.211</v>
+      </c>
+      <c r="G14" t="n">
+        <v>504.791</v>
+      </c>
+      <c r="H14" t="n">
+        <v>71012.33</v>
+      </c>
+      <c r="I14" t="n">
+        <v>18208.379</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-2093.93</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-1.902</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>67</v>
+      </c>
+      <c r="O14" t="n">
+        <v>13.273</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2.564</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất Quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2025-2/2025-04-29/no-name-1745876078.pdf</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:02:43+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BVB</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>115509.397</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6919.239</v>
+      </c>
+      <c r="G15" t="n">
+        <v>643.806</v>
+      </c>
+      <c r="H15" t="n">
+        <v>68796.48299999999</v>
+      </c>
+      <c r="I15" t="n">
+        <v>22013.106</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-11704.532</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-10.133</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-28</v>
+      </c>
+      <c r="O15" t="n">
+        <v>-4.349</v>
+      </c>
+      <c r="P15" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00000617283950617284ngn-hng-tmcp-bn-vit15082025-000000bo-co-ti-chnh-bn-nin-2025_5_1133.pdf</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:53:16+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BVB</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>133047.699</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7460.484</v>
+      </c>
+      <c r="G16" t="n">
+        <v>814.849</v>
+      </c>
+      <c r="H16" t="n">
+        <v>71413.689</v>
+      </c>
+      <c r="I16" t="n">
+        <v>37002.367</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-13892.442</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-10.442</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>5.181</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/_603502_Bao_cao_tai_chinh_nam_2025_1776046380.pdf</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:11:30+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CTG</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2469863.401</v>
+      </c>
+      <c r="F17" t="n">
+        <v>153982.172</v>
+      </c>
+      <c r="G17" t="n">
+        <v>15475.215</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1621227.454</v>
+      </c>
+      <c r="I17" t="n">
+        <v>431140.071</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>148564.507</v>
+      </c>
+      <c r="M17" t="n">
+        <v>6.015</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>2.659</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/CTG_Baocaotaichinh_Q1_2025_Hopnhat_23052025140616.pdf</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:05:00+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CTG</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2609788.006</v>
+      </c>
+      <c r="F18" t="n">
+        <v>163826.196</v>
+      </c>
+      <c r="G18" t="n">
+        <v>15842.616</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1719957.759</v>
+      </c>
+      <c r="I18" t="n">
+        <v>454034.621</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-32156.772</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-1.232</v>
+      </c>
+      <c r="L18" t="n">
+        <v>411358.605</v>
+      </c>
+      <c r="M18" t="n">
+        <v>15.762</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-503</v>
+      </c>
+      <c r="O18" t="n">
+        <v>-3.175</v>
+      </c>
+      <c r="P18" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/CTG_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_03102025145719.pdf</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:55:46+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CTG</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2767699.3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>179655.005</v>
+      </c>
+      <c r="G19" t="n">
+        <v>17959.696</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1793732.057</v>
+      </c>
+      <c r="I19" t="n">
+        <v>524296.557</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-32156.77299999999</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-1.162</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-71057.747</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-2.567</v>
+      </c>
+      <c r="N19" t="n">
+        <v>-503</v>
+      </c>
+      <c r="O19" t="n">
+        <v>-2.801</v>
+      </c>
+      <c r="P19" t="n">
+        <v>2.923</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/CTG_HK_20260331_-_CTG_-_BCTC_hop_nhat_kiem_toan_nam_2025__18062026104622.pdf</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:14:15+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EIB</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>251132.546</v>
+      </c>
+      <c r="F20" t="n">
+        <v>25757.442</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1354.384</v>
+      </c>
+      <c r="H20" t="n">
+        <v>175759.164</v>
+      </c>
+      <c r="I20" t="n">
+        <v>32750.7</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-22896.225</v>
+      </c>
+      <c r="K20" t="n">
+        <v>-9.117000000000001</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-39057.023</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-15.552</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-195</v>
+      </c>
+      <c r="O20" t="n">
+        <v>-14.398</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1.863</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/EIB_Baocaotaichinh_Q1_2025_Hopnhat_22052025162515.pdf</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:06:41+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EIB</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>256441.971</v>
+      </c>
+      <c r="F21" t="n">
+        <v>26067.006</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1469.401</v>
+      </c>
+      <c r="H21" t="n">
+        <v>177345.265</v>
+      </c>
+      <c r="I21" t="n">
+        <v>35038.121</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>5410.181</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1.976</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/EIB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025085527.pdf</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>2026-08-31T11:57:38+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EIB</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>273270.407</v>
+      </c>
+      <c r="F22" t="n">
+        <v>26006.343</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1690.894</v>
+      </c>
+      <c r="H22" t="n">
+        <v>177303.877</v>
+      </c>
+      <c r="I22" t="n">
+        <v>50842.748</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>7930.371999999999</v>
+      </c>
+      <c r="M22" t="n">
+        <v>2.902</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>2.868</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260330_-_EIB_-_BCTC_hop_nhat_nam_2025_da_kiem_toan_1774925122.pdf</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:16:37+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>HDB</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:08:58+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HDB</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:01:17+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HDB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:18:56+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KLB</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>97164.45</v>
+      </c>
+      <c r="F26" t="n">
+        <v>6834.212</v>
+      </c>
+      <c r="G26" t="n">
+        <v>849.086</v>
+      </c>
+      <c r="H26" t="n">
+        <v>70989.97199999999</v>
+      </c>
+      <c r="I26" t="n">
+        <v>18386.133</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>-3996.194</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-4.113</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/000000014864567_VI_BAO_CAO_TAI_CHINH_QUY_I_06052025105844.2025_HOP_NHAT</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:10:19+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KLB</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>97630.48299999999</v>
+      </c>
+      <c r="F27" t="n">
+        <v>7246.143</v>
+      </c>
+      <c r="G27" t="n">
+        <v>883.946</v>
+      </c>
+      <c r="H27" t="n">
+        <v>73173.554</v>
+      </c>
+      <c r="I27" t="n">
+        <v>17449.438</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>33012.88</v>
+      </c>
+      <c r="M27" t="n">
+        <v>33.814</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>2.385</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00000617283950617284ngn-hng-tmcp-kin-long28082025-000000bo-co-ti-chnh-bn-nin-2025_1_0929.pdf</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:03:05+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>KLB</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>103302.689</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8416.503000000001</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1056.67</v>
+      </c>
+      <c r="H28" t="n">
+        <v>72010.409</v>
+      </c>
+      <c r="I28" t="n">
+        <v>22569.94</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2230.823</v>
+      </c>
+      <c r="M28" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>3.134</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260330_-_KLB_-_BCTC_KiemToan_2025_Hop_nhat_1774928715.pdf</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:20:50+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LPB</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:13:34+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LPB</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:07:34+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LPB</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:22:06+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MBB</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1156917.195</v>
+      </c>
+      <c r="F32" t="n">
+        <v>123676.548</v>
+      </c>
+      <c r="G32" t="n">
+        <v>11692.184</v>
+      </c>
+      <c r="H32" t="n">
+        <v>722622.45</v>
+      </c>
+      <c r="I32" t="n">
+        <v>84084.52099999999</v>
+      </c>
+      <c r="J32" t="n">
+        <v>7749.506</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="L32" t="n">
+        <v>183923.188</v>
+      </c>
+      <c r="M32" t="n">
+        <v>15.898</v>
+      </c>
+      <c r="N32" t="n">
+        <v>65</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1.164</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00012345679012345679ngn-hng-tmcp-qun-i24042025-000000bo-co-ti-chnh-hp-nht-qu.pdf</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:15:17+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MBB</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1289644.328</v>
+      </c>
+      <c r="F33" t="n">
+        <v>127803.65</v>
+      </c>
+      <c r="G33" t="n">
+        <v>12372.117</v>
+      </c>
+      <c r="H33" t="n">
+        <v>783291.9080000001</v>
+      </c>
+      <c r="I33" t="n">
+        <v>116595.397</v>
+      </c>
+      <c r="J33" t="n">
+        <v>40113.92999999999</v>
+      </c>
+      <c r="K33" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>-27</v>
+      </c>
+      <c r="O33" t="n">
+        <v>-0.218</v>
+      </c>
+      <c r="P33" t="n">
+        <v>1.489</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/MBB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025091521.pdf</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:10:05+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MBB</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1615763.927</v>
+      </c>
+      <c r="F34" t="n">
+        <v>142022.525</v>
+      </c>
+      <c r="G34" t="n">
+        <v>14555.292</v>
+      </c>
+      <c r="H34" t="n">
+        <v>921368.132</v>
+      </c>
+      <c r="I34" t="n">
+        <v>256383.938</v>
+      </c>
+      <c r="J34" t="n">
+        <v>-119953.924</v>
+      </c>
+      <c r="K34" t="n">
+        <v>-7.424</v>
+      </c>
+      <c r="L34" t="n">
+        <v>-338533.023</v>
+      </c>
+      <c r="M34" t="n">
+        <v>-20.952</v>
+      </c>
+      <c r="N34" t="n">
+        <v>-1506</v>
+      </c>
+      <c r="O34" t="n">
+        <v>-10.347</v>
+      </c>
+      <c r="P34" t="n">
+        <v>2.783</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/MBB_Baocaotaichinh_2025_Kiemtoan_Hopnhat_1780022210.pdf</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:24:23+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>314727.148</v>
+      </c>
+      <c r="F35" t="n">
+        <v>38020.647</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2503.785</v>
+      </c>
+      <c r="H35" t="n">
+        <v>163035.139</v>
+      </c>
+      <c r="I35" t="n">
+        <v>53049.641</v>
+      </c>
+      <c r="J35" t="n">
+        <v>-16352.815</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-5.196</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-71627.23300000001</v>
+      </c>
+      <c r="M35" t="n">
+        <v>-22.759</v>
+      </c>
+      <c r="N35" t="n">
+        <v>-257</v>
+      </c>
+      <c r="O35" t="n">
+        <v>-10.264</v>
+      </c>
+      <c r="P35" t="n">
+        <v>3.254</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00032098765432098763ngn-hng-tmcp-hng-hi-vit-nam28042025-000000bo-co-ti-chnh-hp-nht-qu.pdf</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:17:02+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>341331.296</v>
+      </c>
+      <c r="F36" t="n">
+        <v>39312.119</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2584.839</v>
+      </c>
+      <c r="H36" t="n">
+        <v>174429.9</v>
+      </c>
+      <c r="I36" t="n">
+        <v>64784.029</v>
+      </c>
+      <c r="J36" t="n">
+        <v>88375.88399999999</v>
+      </c>
+      <c r="K36" t="n">
+        <v>25.892</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-78086.85799999999</v>
+      </c>
+      <c r="M36" t="n">
+        <v>-22.877</v>
+      </c>
+      <c r="N36" t="n">
+        <v>774</v>
+      </c>
+      <c r="O36" t="n">
+        <v>29.944</v>
+      </c>
+      <c r="P36" t="n">
+        <v>3.714</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/MSB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025092910.pdf</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:12:00+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>407673.941</v>
+      </c>
+      <c r="F37" t="n">
+        <v>42446.058</v>
+      </c>
+      <c r="G37" t="n">
+        <v>3043.554</v>
+      </c>
+      <c r="H37" t="n">
+        <v>196671.626</v>
+      </c>
+      <c r="I37" t="n">
+        <v>85247.459</v>
+      </c>
+      <c r="J37" t="n">
+        <v>-36336.33499999999</v>
+      </c>
+      <c r="K37" t="n">
+        <v>-8.913</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-94852.075</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-23.267</v>
+      </c>
+      <c r="N37" t="n">
+        <v>-330</v>
+      </c>
+      <c r="O37" t="n">
+        <v>-10.843</v>
+      </c>
+      <c r="P37" t="n">
+        <v>4.335</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/MSB_HK_20260330_-_MSB_-_BCTC_hop_nhat_kiem_toan_nam_2025__18062026110209.pdf</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:26:11+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>NAB</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>262251.025</v>
+      </c>
+      <c r="F38" t="n">
+        <v>20213.631</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2112.162</v>
+      </c>
+      <c r="H38" t="n">
+        <v>176385.625</v>
+      </c>
+      <c r="I38" t="n">
+        <v>53623.62</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1044.137999999999</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-26051.455</v>
+      </c>
+      <c r="M38" t="n">
+        <v>-9.933999999999999</v>
+      </c>
+      <c r="N38" t="n">
+        <v>224</v>
+      </c>
+      <c r="O38" t="n">
+        <v>10.605</v>
+      </c>
+      <c r="P38" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00032098765432098763ngn-hng-tmcp-nam-28042025-000000bo-co-ti-chnh-hp-nht-qu.pdf</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:18:34+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>NAB</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>314798.083</v>
+      </c>
+      <c r="F39" t="n">
+        <v>21239.816</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2122.128</v>
+      </c>
+      <c r="H39" t="n">
+        <v>196932.046</v>
+      </c>
+      <c r="I39" t="n">
+        <v>88326.624</v>
+      </c>
+      <c r="J39" t="n">
+        <v>-7342.066000000003</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-2.332</v>
+      </c>
+      <c r="L39" t="n">
+        <v>-12907.955</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="N39" t="n">
+        <v>140</v>
+      </c>
+      <c r="O39" t="n">
+        <v>6.597</v>
+      </c>
+      <c r="P39" t="n">
+        <v>4.485</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/NAB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025093916.pdf</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:14:18+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NAB</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>418333.322</v>
+      </c>
+      <c r="F40" t="n">
+        <v>23430.767</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2327.558</v>
+      </c>
+      <c r="H40" t="n">
+        <v>177810.693</v>
+      </c>
+      <c r="I40" t="n">
+        <v>170154.001</v>
+      </c>
+      <c r="J40" t="n">
+        <v>506013.917</v>
+      </c>
+      <c r="K40" t="n">
+        <v>120.96</v>
+      </c>
+      <c r="L40" t="n">
+        <v>206015.022</v>
+      </c>
+      <c r="M40" t="n">
+        <v>49.247</v>
+      </c>
+      <c r="N40" t="n">
+        <v>1841</v>
+      </c>
+      <c r="O40" t="n">
+        <v>79.096</v>
+      </c>
+      <c r="P40" t="n">
+        <v>9.569000000000001</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/NAB_Baocaotaichinh_2025_Kiemtoan_Hopnhat_1780023595.pdf</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:28:37+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>NVB</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>130882.914</v>
+      </c>
+      <c r="F41" t="n">
+        <v>6243.613</v>
+      </c>
+      <c r="G41" t="n">
+        <v>504.861</v>
+      </c>
+      <c r="H41" t="n">
+        <v>102527.917</v>
+      </c>
+      <c r="I41" t="n">
+        <v>21312.588</v>
+      </c>
+      <c r="J41" t="n">
+        <v>4928.864</v>
+      </c>
+      <c r="K41" t="n">
+        <v>3.766</v>
+      </c>
+      <c r="L41" t="n">
+        <v>-4695.431</v>
+      </c>
+      <c r="M41" t="n">
+        <v>-3.588</v>
+      </c>
+      <c r="N41" t="n">
+        <v>102</v>
+      </c>
+      <c r="O41" t="n">
+        <v>20.204</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.079</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/NVB_25Q1_BCTC_HN_09052025064513.pdf</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:20:53+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NVB</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>144053.644</v>
+      </c>
+      <c r="F42" t="n">
+        <v>6555.077</v>
+      </c>
+      <c r="G42" t="n">
+        <v>757.676</v>
+      </c>
+      <c r="H42" t="n">
+        <v>115244.771</v>
+      </c>
+      <c r="I42" t="n">
+        <v>25035.067</v>
+      </c>
+      <c r="J42" t="n">
+        <v>-58074.064</v>
+      </c>
+      <c r="K42" t="n">
+        <v>-40.314</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>-319</v>
+      </c>
+      <c r="O42" t="n">
+        <v>-42.102</v>
+      </c>
+      <c r="P42" t="n">
+        <v>2.172</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00000617283950617284ngn-hng-tmcp-quc-dn27082025-000000bo-co-ti-chnh-bn-nin-2025_1_0915.pdf</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:16:11+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NVB</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>163614.988</v>
+      </c>
+      <c r="F43" t="n">
+        <v>13592.924</v>
+      </c>
+      <c r="G43" t="n">
+        <v>423.627</v>
+      </c>
+      <c r="H43" t="n">
+        <v>127403.437</v>
+      </c>
+      <c r="I43" t="n">
+        <v>38989.537</v>
+      </c>
+      <c r="J43" t="n">
+        <v>44447.072</v>
+      </c>
+      <c r="K43" t="n">
+        <v>27.166</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="n">
+        <v>682</v>
+      </c>
+      <c r="O43" t="n">
+        <v>160.991</v>
+      </c>
+      <c r="P43" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/_604185_Bao_cao_tai_chinh_nam_2025_1774532924.pdf</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:30:26+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>OCB</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:23:58+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>OCB</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:23:24+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>OCB</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:30:30+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PGB</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>73551.58199999999</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5242.581</v>
+      </c>
+      <c r="G47" t="n">
+        <v>458.27</v>
+      </c>
+      <c r="H47" t="n">
+        <v>46717.488</v>
+      </c>
+      <c r="I47" t="n">
+        <v>22839.31</v>
+      </c>
+      <c r="J47" t="n">
+        <v>4980.354</v>
+      </c>
+      <c r="K47" t="n">
+        <v>6.771</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="n">
+        <v>35</v>
+      </c>
+      <c r="O47" t="n">
+        <v>7.637</v>
+      </c>
+      <c r="P47" t="n">
+        <v>4.889</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất Quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2025-2/2025-04-18/no-name-1744937049.pdf</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:25:19+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PGB</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>78533.89999999999</v>
+      </c>
+      <c r="F48" t="n">
+        <v>6177.553</v>
+      </c>
+      <c r="G48" t="n">
+        <v>471.899</v>
+      </c>
+      <c r="H48" t="n">
+        <v>46726.281</v>
+      </c>
+      <c r="I48" t="n">
+        <v>24930.12</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1419.186</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.807</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-3100.088</v>
+      </c>
+      <c r="M48" t="n">
+        <v>-3.947</v>
+      </c>
+      <c r="N48" t="n">
+        <v>4</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="P48" t="n">
+        <v>5.335</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất Quý 2 năm 2025</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2025-3/2025-08-19/no-name-1755541972.pdf</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:25:04+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PGB</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>88840.17200000001</v>
+      </c>
+      <c r="F49" t="n">
+        <v>6545.253</v>
+      </c>
+      <c r="G49" t="n">
+        <v>481.771</v>
+      </c>
+      <c r="H49" t="n">
+        <v>48460.417</v>
+      </c>
+      <c r="I49" t="n">
+        <v>31153.789</v>
+      </c>
+      <c r="J49" t="n">
+        <v>-448.712</v>
+      </c>
+      <c r="K49" t="n">
+        <v>-0.505</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-7944.858999999999</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-8.943</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-20</v>
+      </c>
+      <c r="O49" t="n">
+        <v>-4.151</v>
+      </c>
+      <c r="P49" t="n">
+        <v>6.429</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất đã kiểm toán năm 2025</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2026-2/2026-04-02/no-name-1775069400.pdf</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:31:51+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SGB</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>33506.33</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4172.432</v>
+      </c>
+      <c r="G50" t="n">
+        <v>217.861</v>
+      </c>
+      <c r="H50" t="n">
+        <v>24539.598</v>
+      </c>
+      <c r="I50" t="n">
+        <v>9035.235999999999</v>
+      </c>
+      <c r="J50" t="n">
+        <v>-8415.234000000002</v>
+      </c>
+      <c r="K50" t="n">
+        <v>-25.115</v>
+      </c>
+      <c r="L50" t="n">
+        <v>5121.561</v>
+      </c>
+      <c r="M50" t="n">
+        <v>15.285</v>
+      </c>
+      <c r="N50" t="n">
+        <v>-102</v>
+      </c>
+      <c r="O50" t="n">
+        <v>-46.819</v>
+      </c>
+      <c r="P50" t="n">
+        <v>3.682</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/000000014834796_VI_BaoCaotaiChinh_HopNhat_Q1_2025_26042025110134.pdf</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:26:54+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>SGB</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>35140.737</v>
+      </c>
+      <c r="F51" t="n">
+        <v>4234.018</v>
+      </c>
+      <c r="G51" t="n">
+        <v>233.402</v>
+      </c>
+      <c r="H51" t="n">
+        <v>25595.19</v>
+      </c>
+      <c r="I51" t="n">
+        <v>10508.501</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1423.367</v>
+      </c>
+      <c r="K51" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="L51" t="n">
+        <v>1633.754</v>
+      </c>
+      <c r="M51" t="n">
+        <v>4.649</v>
+      </c>
+      <c r="N51" t="n">
+        <v>-14</v>
+      </c>
+      <c r="O51" t="n">
+        <v>-5.998</v>
+      </c>
+      <c r="P51" t="n">
+        <v>4.106</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00019753086419753087ngn-hng-tmcp-si-gn-cng-thng14082025-000000bo-co-ti-chnh-bn-nin-2025_1_1022.pdf</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:26:51+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SGB</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>35377.029</v>
+      </c>
+      <c r="F52" t="n">
+        <v>4194.143</v>
+      </c>
+      <c r="G52" t="n">
+        <v>65.943</v>
+      </c>
+      <c r="H52" t="n">
+        <v>26326.61</v>
+      </c>
+      <c r="I52" t="n">
+        <v>9373.537</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3391.897</v>
+      </c>
+      <c r="K52" t="n">
+        <v>9.587999999999999</v>
+      </c>
+      <c r="L52" t="n">
+        <v>838.0600000000001</v>
+      </c>
+      <c r="M52" t="n">
+        <v>2.369</v>
+      </c>
+      <c r="N52" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O52" t="n">
+        <v>-10.615</v>
+      </c>
+      <c r="P52" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/_604675_Bao_cao_tai_chinh_nam_2025_1776046299.pdf</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:33:44+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SHB</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:28:16+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>SHB</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>825718.9790000001</v>
+      </c>
+      <c r="F54" t="n">
+        <v>63267.914</v>
+      </c>
+      <c r="G54" t="n">
+        <v>9160.064</v>
+      </c>
+      <c r="H54" t="n">
+        <v>561718.311</v>
+      </c>
+      <c r="I54" t="n">
+        <v>139362.736</v>
+      </c>
+      <c r="J54" t="n">
+        <v>101052.076</v>
+      </c>
+      <c r="K54" t="n">
+        <v>12.238</v>
+      </c>
+      <c r="L54" t="n">
+        <v>7001.849</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="N54" t="n">
+        <v>1186</v>
+      </c>
+      <c r="O54" t="n">
+        <v>12.948</v>
+      </c>
+      <c r="P54" t="n">
+        <v>2.481</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20250903_-_SHB_-_Bao_Cao_Tai_Chinh_Hop_Nhat_Soat_Xet_Ban_nien_30.6.2025_1756910753.pdf</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:28:17+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>SHB</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:34:56+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SSB</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>333746.268</v>
+      </c>
+      <c r="F56" t="n">
+        <v>38599.606</v>
+      </c>
+      <c r="G56" t="n">
+        <v>2450.482</v>
+      </c>
+      <c r="H56" t="n">
+        <v>160043.132</v>
+      </c>
+      <c r="I56" t="n">
+        <v>83940.10000000001</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="n">
+        <v>24719.945</v>
+      </c>
+      <c r="M56" t="n">
+        <v>7.407</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" t="n">
+        <v>5.245</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/SSB_23052025144847.pdf</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:31:02+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SSB</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>379013.742</v>
+      </c>
+      <c r="F57" t="n">
+        <v>39487.97</v>
+      </c>
+      <c r="G57" t="n">
+        <v>2464.389</v>
+      </c>
+      <c r="H57" t="n">
+        <v>166648.051</v>
+      </c>
+      <c r="I57" t="n">
+        <v>117396.389</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="n">
+        <v>26000.343</v>
+      </c>
+      <c r="M57" t="n">
+        <v>6.86</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" t="n">
+        <v>7.045</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20250905_-_SSB_-_Bao_cao_tai_chinh_hop_nhat_soat_xet_ban_nien_2025_va_Giai_trinh_bien_dong_LNST_signed_1757323427.pdf</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:30:19+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SSB</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>396443.131</v>
+      </c>
+      <c r="F58" t="n">
+        <v>40372.594</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2451.866</v>
+      </c>
+      <c r="H58" t="n">
+        <v>191807.215</v>
+      </c>
+      <c r="I58" t="n">
+        <v>116960.044</v>
+      </c>
+      <c r="J58" t="n">
+        <v>25542.62000000001</v>
+      </c>
+      <c r="K58" t="n">
+        <v>6.443</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1371.248</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="N58" t="n">
+        <v>568</v>
+      </c>
+      <c r="O58" t="n">
+        <v>23.166</v>
+      </c>
+      <c r="P58" t="n">
+        <v>6.098</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260312_-_SSB_-_BCTC_hop_nhat_kiem_toan_nam_2025_kem_Giai_trinh_bien_dong_LNST_signed_1773310402.pdf</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:36:28+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>STB</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>757093.326</v>
+      </c>
+      <c r="F59" t="n">
+        <v>57862.377</v>
+      </c>
+      <c r="G59" t="n">
+        <v>6863.173</v>
+      </c>
+      <c r="H59" t="n">
+        <v>585569.336</v>
+      </c>
+      <c r="I59" t="n">
+        <v>100730.034</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
+        <v>8816.550999999999</v>
+      </c>
+      <c r="M59" t="n">
+        <v>1.165</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00032098765432098763ngn-hng-tmcp-si-gn-thng-tn26042025-000000bo-co-ti-chnh-hp-nht-qu.pdf</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:34:12+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>STB</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>807339.224</v>
+      </c>
+      <c r="F60" t="n">
+        <v>59821.207</v>
+      </c>
+      <c r="G60" t="n">
+        <v>6585.077</v>
+      </c>
+      <c r="H60" t="n">
+        <v>624314.777</v>
+      </c>
+      <c r="I60" t="n">
+        <v>125819.938</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="n">
+        <v>-70865.32000000001</v>
+      </c>
+      <c r="M60" t="n">
+        <v>-8.778</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="n">
+        <v>2.015</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/STB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025100208.pdf</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:33:00+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>STB</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>917119.803</v>
+      </c>
+      <c r="F61" t="n">
+        <v>59866.744</v>
+      </c>
+      <c r="G61" t="n">
+        <v>5358.002</v>
+      </c>
+      <c r="H61" t="n">
+        <v>618341.672</v>
+      </c>
+      <c r="I61" t="n">
+        <v>195970.826</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
+        <v>-147426.407</v>
+      </c>
+      <c r="M61" t="n">
+        <v>-16.075</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>3.169</v>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260327_-_STB_-_BCTC_Hop_nhat_nam_2025_da_kiem_toan__1774863040.pdf</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:38:47+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TCB</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>989215.993</v>
+      </c>
+      <c r="F62" t="n">
+        <v>153952.665</v>
+      </c>
+      <c r="G62" t="n">
+        <v>8305.393</v>
+      </c>
+      <c r="H62" t="n">
+        <v>531583.052</v>
+      </c>
+      <c r="I62" t="n">
+        <v>148372.369</v>
+      </c>
+      <c r="J62" t="n">
+        <v>12025.473</v>
+      </c>
+      <c r="K62" t="n">
+        <v>1.216</v>
+      </c>
+      <c r="L62" t="n">
+        <v>-28602.92</v>
+      </c>
+      <c r="M62" t="n">
+        <v>-2.891</v>
+      </c>
+      <c r="N62" t="n">
+        <v>-470</v>
+      </c>
+      <c r="O62" t="n">
+        <v>-5.659</v>
+      </c>
+      <c r="P62" t="n">
+        <v>2.791</v>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00001234567901234568ngn-hng-tmcp-k-thng-vit-nam21042025-000000bo-co-ti-chnh-hp-nht-qu.pdf</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:35:54+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TCB</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1037645.395</v>
+      </c>
+      <c r="F63" t="n">
+        <v>161827.229</v>
+      </c>
+      <c r="G63" t="n">
+        <v>9137.075999999999</v>
+      </c>
+      <c r="H63" t="n">
+        <v>545078.843</v>
+      </c>
+      <c r="I63" t="n">
+        <v>132997.785</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="n">
+        <v>-64704.99100000001</v>
+      </c>
+      <c r="M63" t="n">
+        <v>-6.236</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/TCB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025101639.pdf</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:36:30+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TCB</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1192344.137</v>
+      </c>
+      <c r="F64" t="n">
+        <v>179501.442</v>
+      </c>
+      <c r="G64" t="n">
+        <v>10787.979</v>
+      </c>
+      <c r="H64" t="n">
+        <v>618911.535</v>
+      </c>
+      <c r="I64" t="n">
+        <v>201481.905</v>
+      </c>
+      <c r="J64" t="n">
+        <v>-95355.82799999998</v>
+      </c>
+      <c r="K64" t="n">
+        <v>-7.997</v>
+      </c>
+      <c r="L64" t="n">
+        <v>-31183.875</v>
+      </c>
+      <c r="M64" t="n">
+        <v>-2.615</v>
+      </c>
+      <c r="N64" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="O64" t="n">
+        <v>-9.27</v>
+      </c>
+      <c r="P64" t="n">
+        <v>3.255</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260317_-_TCB_-_Techcombank-VAS-bao_cao_tai_chinh_hop_nhat-YE25_1773755161.pdf</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:41:25+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>TPB</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:40:47+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>TPB</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:42:52+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>TPB</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>505901.57</v>
+      </c>
+      <c r="F67" t="n">
+        <v>46048.761</v>
+      </c>
+      <c r="G67" t="n">
+        <v>3598.599</v>
+      </c>
+      <c r="H67" t="n">
+        <v>279050.251</v>
+      </c>
+      <c r="I67" t="n">
+        <v>125552.772</v>
+      </c>
+      <c r="J67" t="n">
+        <v>1.704</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="n">
+        <v>4.499</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260331_-_TPB_-_BCTC_hop_nhat_2025_da_kiem_toan_kem_giai_trinh_chenh_lech_LNST_signed_1774952109.pdf</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:43:30+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>VAB</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>129046.444409199</v>
+      </c>
+      <c r="F68" t="n">
+        <v>9151.860456363</v>
+      </c>
+      <c r="G68" t="n">
+        <v>612.5349521319999</v>
+      </c>
+      <c r="H68" t="n">
+        <v>93896.377376687</v>
+      </c>
+      <c r="I68" t="n">
+        <v>19187.7140786</v>
+      </c>
+      <c r="J68" t="n">
+        <v>26350.65</v>
+      </c>
+      <c r="K68" t="n">
+        <v>20.42</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>167</v>
+      </c>
+      <c r="O68" t="n">
+        <v>27.264</v>
+      </c>
+      <c r="P68" t="n">
+        <v>2.043</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/000000014787653_VI_BaoCaoTaiChinh_Q1_2025_18042025134138.pdf</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:42:19+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>VAB</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:46:28+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>VAB</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>140485.531667485</v>
+      </c>
+      <c r="F70" t="n">
+        <v>10155.027138318</v>
+      </c>
+      <c r="G70" t="n">
+        <v>1608.289139551</v>
+      </c>
+      <c r="H70" t="n">
+        <v>99079.937892602</v>
+      </c>
+      <c r="I70" t="n">
+        <v>23789.312582522</v>
+      </c>
+      <c r="J70" t="n">
+        <v>9801.561999999998</v>
+      </c>
+      <c r="K70" t="n">
+        <v>6.977</v>
+      </c>
+      <c r="L70" t="n">
+        <v>11145.647</v>
+      </c>
+      <c r="M70" t="n">
+        <v>7.934</v>
+      </c>
+      <c r="N70" t="n">
+        <v>114</v>
+      </c>
+      <c r="O70" t="n">
+        <v>7.088</v>
+      </c>
+      <c r="P70" t="n">
+        <v>2.401</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260330_-_VAB_BCTC_hop_nhat_da_kiem_toan_Nam_2025_1775054500.pdf</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:45:19+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>VBB</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>174377.72</v>
+      </c>
+      <c r="F71" t="n">
+        <v>8897.989</v>
+      </c>
+      <c r="G71" t="n">
+        <v>702.5119999999999</v>
+      </c>
+      <c r="H71" t="n">
+        <v>103017.174</v>
+      </c>
+      <c r="I71" t="n">
+        <v>49825.872</v>
+      </c>
+      <c r="J71" t="n">
+        <v>14256.841</v>
+      </c>
+      <c r="K71" t="n">
+        <v>8.176</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>51</v>
+      </c>
+      <c r="O71" t="n">
+        <v>7.26</v>
+      </c>
+      <c r="P71" t="n">
+        <v>4.837</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/1_vbb_2025_5_7_121b03c_vi_baocaotaichinh_hopnhat_q1_20251_16052025112437.pdf</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:44:04+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>VBB</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>178670.984</v>
+      </c>
+      <c r="F72" t="n">
+        <v>9073.486999999999</v>
+      </c>
+      <c r="G72" t="n">
+        <v>687.4059999999999</v>
+      </c>
+      <c r="H72" t="n">
+        <v>104208.415</v>
+      </c>
+      <c r="I72" t="n">
+        <v>45431.683</v>
+      </c>
+      <c r="J72" t="n">
+        <v>16300.747</v>
+      </c>
+      <c r="K72" t="n">
+        <v>9.122999999999999</v>
+      </c>
+      <c r="L72" t="n">
+        <v>-3955.115</v>
+      </c>
+      <c r="M72" t="n">
+        <v>-2.214</v>
+      </c>
+      <c r="N72" t="n">
+        <v>143</v>
+      </c>
+      <c r="O72" t="n">
+        <v>20.803</v>
+      </c>
+      <c r="P72" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00015520282186948853ngn-hng-tmcp-vit-nam-thng-tn05082025-000000bo-co-ti-chnh-bn-nin-2025_1_1517.pdf</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:48:36+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>VBB</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>196771.033</v>
+      </c>
+      <c r="F73" t="n">
+        <v>12431.567</v>
+      </c>
+      <c r="G73" t="n">
+        <v>1108.674</v>
+      </c>
+      <c r="H73" t="n">
+        <v>101449.573</v>
+      </c>
+      <c r="I73" t="n">
+        <v>56200.61</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" t="n">
+        <v>-8211.225</v>
+      </c>
+      <c r="M73" t="n">
+        <v>-4.173</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/_603183_Bao_cao_tai_chinh_nam_2025_1776046427.pdf</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:48:14+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>VCB</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:46:39+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>VCB</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2217636.6</v>
+      </c>
+      <c r="F75" t="n">
+        <v>213749.422</v>
+      </c>
+      <c r="G75" t="n">
+        <v>14160.192</v>
+      </c>
+      <c r="H75" t="n">
+        <v>1586682.675</v>
+      </c>
+      <c r="I75" t="n">
+        <v>485017.633</v>
+      </c>
+      <c r="J75" t="n">
+        <v>-43033.196</v>
+      </c>
+      <c r="K75" t="n">
+        <v>-1.94</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" t="n">
+        <v>-487</v>
+      </c>
+      <c r="O75" t="n">
+        <v>-3.439</v>
+      </c>
+      <c r="P75" t="n">
+        <v>3.057</v>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/VCB_Baocaotaichinh_6T_2025_Soatxet_Hopnhat_06102025111259.pdf</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:50:26+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>VCB</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>2442279.166</v>
+      </c>
+      <c r="F76" t="n">
+        <v>224558.726</v>
+      </c>
+      <c r="G76" t="n">
+        <v>16266.825</v>
+      </c>
+      <c r="H76" t="n">
+        <v>1672534.846</v>
+      </c>
+      <c r="I76" t="n">
+        <v>575462.635</v>
+      </c>
+      <c r="J76" t="n">
+        <v>819.975</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>7</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="P76" t="n">
+        <v>3.441</v>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260327_-_VCB_-_BCTC_hop_nhat_kiem_toan_nam_2025_1774870712.pdf</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:50:20+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>VIB</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2025-Q1</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>495727.377</v>
+      </c>
+      <c r="F77" t="n">
+        <v>43643.267</v>
+      </c>
+      <c r="G77" t="n">
+        <v>3737.109</v>
+      </c>
+      <c r="H77" t="n">
+        <v>282298.036</v>
+      </c>
+      <c r="I77" t="n">
+        <v>109632.918</v>
+      </c>
+      <c r="J77" t="n">
+        <v>60162.859</v>
+      </c>
+      <c r="K77" t="n">
+        <v>12.136</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" t="n">
+        <v>370</v>
+      </c>
+      <c r="O77" t="n">
+        <v>9.901</v>
+      </c>
+      <c r="P77" t="n">
+        <v>3.884</v>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất đã kiểm toán Quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2025-3/2025-07-29/no-name-1753727617.pdf</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:48:45+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>VIB</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2025-Q2</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>530909.024</v>
+      </c>
+      <c r="F78" t="n">
+        <v>43627.741</v>
+      </c>
+      <c r="G78" t="n">
+        <v>3968.694</v>
+      </c>
+      <c r="H78" t="n">
+        <v>304392.951</v>
+      </c>
+      <c r="I78" t="n">
+        <v>104990.528</v>
+      </c>
+      <c r="J78" t="n">
+        <v>50291.15800000001</v>
+      </c>
+      <c r="K78" t="n">
+        <v>9.473000000000001</v>
+      </c>
+      <c r="L78" t="n">
+        <v>-74107.53099999999</v>
+      </c>
+      <c r="M78" t="n">
+        <v>-13.959</v>
+      </c>
+      <c r="N78" t="n">
+        <v>-130</v>
+      </c>
+      <c r="O78" t="n">
+        <v>-3.276</v>
+      </c>
+      <c r="P78" t="n">
+        <v>3.449</v>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 2 năm 2025 (đã soát xét)</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/00015520282186948853ngn-hng-tmcp-quc-t-vit-nam06082025-000000bo-co-ti-chnh-hp-nht-bn-nin_1_0929.pdf</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>2026-08-31T12:52:16+07:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>VIB</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2025-FY</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>556098.441</v>
+      </c>
+      <c r="F79" t="n">
+        <v>46904.739</v>
+      </c>
+      <c r="G79" t="n">
+        <v>4213.631</v>
+      </c>
+      <c r="H79" t="n">
+        <v>294577.661</v>
+      </c>
+      <c r="I79" t="n">
+        <v>116961.762</v>
+      </c>
+      <c r="J79" t="n">
+        <v>26608.905</v>
+      </c>
+      <c r="K79" t="n">
+        <v>4.785</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>-278</v>
+      </c>
+      <c r="O79" t="n">
+        <v>-6.598</v>
+      </c>
+      <c r="P79" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất năm 2025 (đã kiểm toán)</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/20260302_-_VIB_-_BCTC_hop_nhat_kiem_toan_2025_1772443477.pdf</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:52:28+07:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Backfill ALM ngan hang — 2025-Q1 — 2026-08-31
</commit_message>
<xml_diff>
--- a/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
+++ b/Bao cao/VIMO/VIMO_Lich_Su_Chi_So.xlsx
@@ -31280,7 +31280,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>2026-08-31T10:01:27+07:00</t>
+          <t>2026-08-31T16:51:48+07:00</t>
         </is>
       </c>
     </row>
@@ -32566,12 +32566,94 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>711310.758</v>
+      </c>
+      <c r="F30" t="n">
+        <v>61032.537</v>
+      </c>
+      <c r="G30" t="n">
+        <v>7408.1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>465321.208</v>
+      </c>
+      <c r="I30" t="n">
+        <v>440468.264</v>
+      </c>
+      <c r="J30" t="n">
+        <v>94.65900000000001</v>
+      </c>
+      <c r="K30" t="n">
+        <v>148462.094</v>
+      </c>
+      <c r="L30" t="n">
+        <v>103248.139</v>
+      </c>
+      <c r="M30" t="n">
+        <v>14.515</v>
+      </c>
+      <c r="N30" t="n">
+        <v>20.753</v>
+      </c>
+      <c r="O30" t="n">
+        <v>33.588</v>
+      </c>
+      <c r="P30" t="n">
+        <v>190653.82</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>22959.914</v>
+      </c>
+      <c r="R30" t="n">
+        <v>830.377</v>
+      </c>
+      <c r="S30" t="n">
+        <v>419.939</v>
+      </c>
+      <c r="T30" t="n">
+        <v>23.813</v>
+      </c>
+      <c r="U30" t="n">
+        <v>3.191</v>
+      </c>
+      <c r="V30" t="n">
+        <v>104881.84</v>
+      </c>
+      <c r="W30" t="n">
+        <v>-10.601</v>
+      </c>
+      <c r="X30" t="n">
+        <v>-4.327</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>14.745</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>155</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>2.092</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/HDB_23052025143646.pdf</t>
         </is>
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>2026-08-31T10:08:58+07:00</t>
+          <t>2026-08-31T16:53:47+07:00</t>
         </is>
       </c>
     </row>
@@ -33070,12 +33152,94 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>499894.623</v>
+      </c>
+      <c r="F38" t="n">
+        <v>45872.206</v>
+      </c>
+      <c r="G38" t="n">
+        <v>3281.91</v>
+      </c>
+      <c r="H38" t="n">
+        <v>293154.504</v>
+      </c>
+      <c r="I38" t="n">
+        <v>347669.189</v>
+      </c>
+      <c r="J38" t="n">
+        <v>118.596</v>
+      </c>
+      <c r="K38" t="n">
+        <v>80298.76300000001</v>
+      </c>
+      <c r="L38" t="n">
+        <v>3081.205</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="N38" t="n">
+        <v>-11.673</v>
+      </c>
+      <c r="O38" t="n">
+        <v>-16.57</v>
+      </c>
+      <c r="P38" t="n">
+        <v>67604.304</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>176873.865</v>
+      </c>
+      <c r="R38" t="n">
+        <v>38.222</v>
+      </c>
+      <c r="S38" t="n">
+        <v>77.506</v>
+      </c>
+      <c r="T38" t="n">
+        <v>129.022</v>
+      </c>
+      <c r="U38" t="n">
+        <v>2.739</v>
+      </c>
+      <c r="V38" t="n">
+        <v>0</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất Quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>https://cdn.24hmoney.vn/upload/file/2025-3/2025-07-22/no-name-1753123076.pdf</t>
         </is>
       </c>
       <c r="AH38" t="inlineStr">
         <is>
-          <t>2026-08-31T10:13:34+07:00</t>
+          <t>2026-08-31T16:55:44+07:00</t>
         </is>
       </c>
     </row>
@@ -34849,7 +35013,7 @@
       </c>
       <c r="AH58" t="inlineStr">
         <is>
-          <t>2026-08-31T10:23:58+07:00</t>
+          <t>2026-08-31T16:58:48+07:00</t>
         </is>
       </c>
     </row>
@@ -35694,7 +35858,7 @@
       </c>
       <c r="AH70" t="inlineStr">
         <is>
-          <t>2026-08-31T10:28:16+07:00</t>
+          <t>2026-08-31T17:00:11+07:00</t>
         </is>
       </c>
     </row>
@@ -37052,7 +37216,7 @@
       </c>
       <c r="AH86" t="inlineStr">
         <is>
-          <t>2026-08-31T10:40:47+07:00</t>
+          <t>2026-08-31T17:05:53+07:00</t>
         </is>
       </c>
     </row>
@@ -37825,12 +37989,94 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>missing</t>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>2109260.616</v>
+      </c>
+      <c r="F98" t="n">
+        <v>204941.834</v>
+      </c>
+      <c r="G98" t="n">
+        <v>13687.153</v>
+      </c>
+      <c r="H98" t="n">
+        <v>1509113.389</v>
+      </c>
+      <c r="I98" t="n">
+        <v>1433896.493</v>
+      </c>
+      <c r="J98" t="n">
+        <v>95.01600000000001</v>
+      </c>
+      <c r="K98" t="n">
+        <v>452321.798</v>
+      </c>
+      <c r="L98" t="n">
+        <v>-461316.069</v>
+      </c>
+      <c r="M98" t="n">
+        <v>-21.871</v>
+      </c>
+      <c r="N98" t="n">
+        <v>-14.033</v>
+      </c>
+      <c r="O98" t="n">
+        <v>-11.763</v>
+      </c>
+      <c r="P98" t="n">
+        <v>1888113.608</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>502117.121</v>
+      </c>
+      <c r="R98" t="n">
+        <v>376.031</v>
+      </c>
+      <c r="S98" t="n">
+        <v>44.043</v>
+      </c>
+      <c r="T98" t="n">
+        <v>227.051</v>
+      </c>
+      <c r="U98" t="n">
+        <v>2.997</v>
+      </c>
+      <c r="V98" t="n">
+        <v>-16699.62499999997</v>
+      </c>
+      <c r="W98" t="n">
+        <v>-17.035</v>
+      </c>
+      <c r="X98" t="n">
+        <v>-2.394</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>-0.792</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>-118</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>-0.862</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>-0.058</v>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính hợp nhất quý 1 năm 2025</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>https://cafefnew.mediacdn.vn/Images/Uploaded/DuLieuDownload/BCTC/VCB_23052025150224.pdf</t>
         </is>
       </c>
       <c r="AH98" t="inlineStr">
         <is>
-          <t>2026-08-31T10:46:39+07:00</t>
+          <t>2026-08-31T17:07:33+07:00</t>
         </is>
       </c>
     </row>

</xml_diff>